<commit_message>
PCB work on out of board connections
</commit_message>
<xml_diff>
--- a/tool/ESP32_Pinout.xlsx
+++ b/tool/ESP32_Pinout.xlsx
@@ -5,18 +5,17 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\myspa\Projects\SEED25\tool\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Files_NK\Projects\SEED25\tool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF0E90BE-A763-425B-B25F-DCFAA9AE1142}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E30887A0-D381-4795-A5B3-D34D74A3700B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="1695" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -26,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="72">
   <si>
     <t>ESP32 Devkit V1 30 pin</t>
   </si>
@@ -139,9 +138,6 @@
     <t>D19</t>
   </si>
   <si>
-    <t>Input Only</t>
-  </si>
-  <si>
     <t>Must be high for boot and low for programming</t>
   </si>
   <si>
@@ -187,9 +183,6 @@
     <t>Tool stepper step</t>
   </si>
   <si>
-    <t>Bump Switch input</t>
-  </si>
-  <si>
     <t>NA</t>
   </si>
   <si>
@@ -233,6 +226,21 @@
   </si>
   <si>
     <t>HB 2</t>
+  </si>
+  <si>
+    <t>(ALT) Step Step</t>
+  </si>
+  <si>
+    <t>(ALT) Step dir</t>
+  </si>
+  <si>
+    <t>(ALT) Step en</t>
+  </si>
+  <si>
+    <t>Home Switch input</t>
+  </si>
+  <si>
+    <t>Input Only (NO PULLUP!)</t>
   </si>
 </sst>
 </file>
@@ -763,20 +771,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G40"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="29.15625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="13.83984375" customWidth="1"/>
-    <col min="6" max="6" width="5.3671875" customWidth="1"/>
-    <col min="7" max="7" width="19.5234375" customWidth="1"/>
+    <col min="4" max="4" width="29.140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="13.85546875" customWidth="1"/>
+    <col min="6" max="6" width="5.42578125" customWidth="1"/>
+    <col min="7" max="7" width="19.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="14.7" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="1" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="43.5" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="2" spans="1:7" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="15" t="s">
         <v>1</v>
       </c>
@@ -790,16 +798,16 @@
         <v>4</v>
       </c>
       <c r="E2" s="16" t="s">
+        <v>45</v>
+      </c>
+      <c r="F2" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="G2" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="F2" s="17" t="s">
-        <v>59</v>
-      </c>
-      <c r="G2" s="18" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+    </row>
+    <row r="3" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
         <v>5</v>
       </c>
@@ -808,15 +816,15 @@
       </c>
       <c r="C3" s="12"/>
       <c r="D3" s="13" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E3" s="14"/>
       <c r="F3" s="11" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="G3" s="11"/>
     </row>
-    <row r="4" spans="1:7" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
@@ -825,15 +833,15 @@
       </c>
       <c r="C4" s="5"/>
       <c r="D4" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E4" s="10"/>
       <c r="F4" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>7</v>
       </c>
@@ -842,15 +850,15 @@
       </c>
       <c r="C5" s="4"/>
       <c r="D5" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E5" s="10"/>
       <c r="F5" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>8</v>
       </c>
@@ -859,15 +867,15 @@
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E6" s="10"/>
       <c r="F6" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>9</v>
       </c>
@@ -878,13 +886,13 @@
       <c r="D7" s="3"/>
       <c r="E7" s="10"/>
       <c r="F7" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
@@ -893,15 +901,15 @@
       </c>
       <c r="C8" s="4"/>
       <c r="D8" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E8" s="10"/>
       <c r="F8" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="G8" s="2"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
         <v>11</v>
       </c>
@@ -910,15 +918,15 @@
       </c>
       <c r="C9" s="8"/>
       <c r="D9" s="9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E9" s="10"/>
       <c r="F9" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G9" s="2"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
         <v>12</v>
       </c>
@@ -927,15 +935,15 @@
       </c>
       <c r="C10" s="8"/>
       <c r="D10" s="9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E10" s="10"/>
       <c r="F10" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G10" s="2"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
         <v>13</v>
       </c>
@@ -944,15 +952,15 @@
       </c>
       <c r="C11" s="8"/>
       <c r="D11" s="9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E11" s="10"/>
       <c r="F11" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G11" s="2"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
         <v>14</v>
       </c>
@@ -961,15 +969,15 @@
       </c>
       <c r="C12" s="8"/>
       <c r="D12" s="9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E12" s="10"/>
       <c r="F12" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G12" s="2"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
         <v>15</v>
       </c>
@@ -978,15 +986,15 @@
       </c>
       <c r="C13" s="8"/>
       <c r="D13" s="9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E13" s="10"/>
       <c r="F13" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G13" s="2"/>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
         <v>16</v>
       </c>
@@ -995,15 +1003,15 @@
       </c>
       <c r="C14" s="8"/>
       <c r="D14" s="9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E14" s="10"/>
       <c r="F14" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G14" s="2"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>17</v>
       </c>
@@ -1012,15 +1020,15 @@
       </c>
       <c r="C15" s="4"/>
       <c r="D15" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E15" s="10"/>
       <c r="F15" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G15" s="2"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>18</v>
       </c>
@@ -1031,11 +1039,11 @@
       <c r="D16" s="3"/>
       <c r="E16" s="10"/>
       <c r="F16" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G16" s="2"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>19</v>
       </c>
@@ -1046,11 +1054,11 @@
       <c r="D17" s="3"/>
       <c r="E17" s="10"/>
       <c r="F17" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G17" s="2"/>
     </row>
-    <row r="18" spans="1:7" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>20</v>
       </c>
@@ -1059,15 +1067,15 @@
       </c>
       <c r="C18" s="4"/>
       <c r="D18" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E18" s="10"/>
       <c r="F18" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G18" s="2"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>22</v>
       </c>
@@ -1078,11 +1086,13 @@
       <c r="D19" s="3"/>
       <c r="E19" s="10"/>
       <c r="F19" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="G19" s="2"/>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>55</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>23</v>
       </c>
@@ -1093,11 +1103,13 @@
       <c r="D20" s="3"/>
       <c r="E20" s="10"/>
       <c r="F20" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="G20" s="2"/>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>55</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>21</v>
       </c>
@@ -1108,13 +1120,13 @@
       <c r="D21" s="3"/>
       <c r="E21" s="10"/>
       <c r="F21" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>36</v>
       </c>
@@ -1125,13 +1137,13 @@
       <c r="D22" s="3"/>
       <c r="E22" s="10"/>
       <c r="F22" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>24</v>
       </c>
@@ -1141,16 +1153,16 @@
       <c r="C23" s="6"/>
       <c r="D23" s="3"/>
       <c r="E23" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="G23" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="F23" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>25</v>
       </c>
@@ -1160,16 +1172,16 @@
       <c r="C24" s="6"/>
       <c r="D24" s="3"/>
       <c r="E24" s="10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>26</v>
       </c>
@@ -1180,13 +1192,13 @@
       <c r="D25" s="3"/>
       <c r="E25" s="10"/>
       <c r="F25" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>27</v>
       </c>
@@ -1197,11 +1209,13 @@
       <c r="D26" s="3"/>
       <c r="E26" s="10"/>
       <c r="F26" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="G26" s="2"/>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>61</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>28</v>
       </c>
@@ -1212,13 +1226,13 @@
       <c r="D27" s="3"/>
       <c r="E27" s="10"/>
       <c r="F27" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>29</v>
       </c>
@@ -1229,13 +1243,13 @@
       <c r="D28" s="3"/>
       <c r="E28" s="10"/>
       <c r="F28" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>30</v>
       </c>
@@ -1246,13 +1260,13 @@
       <c r="D29" s="3"/>
       <c r="E29" s="10"/>
       <c r="F29" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>31</v>
       </c>
@@ -1263,13 +1277,13 @@
       <c r="D30" s="3"/>
       <c r="E30" s="10"/>
       <c r="F30" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>32</v>
       </c>
@@ -1278,15 +1292,15 @@
       </c>
       <c r="C31" s="4"/>
       <c r="D31" s="3" t="s">
-        <v>37</v>
+        <v>71</v>
       </c>
       <c r="E31" s="10"/>
       <c r="F31" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="G31" s="2"/>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>33</v>
       </c>
@@ -1295,15 +1309,15 @@
       </c>
       <c r="C32" s="4"/>
       <c r="D32" s="3" t="s">
-        <v>37</v>
+        <v>71</v>
       </c>
       <c r="E32" s="10"/>
       <c r="F32" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="G32" s="2"/>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>34</v>
       </c>
@@ -1312,15 +1326,15 @@
       </c>
       <c r="C33" s="4"/>
       <c r="D33" s="3" t="s">
-        <v>37</v>
+        <v>71</v>
       </c>
       <c r="E33" s="10"/>
       <c r="F33" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="G33" s="2"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>35</v>
       </c>
@@ -1329,33 +1343,33 @@
       </c>
       <c r="C34" s="4"/>
       <c r="D34" s="3" t="s">
-        <v>37</v>
+        <v>71</v>
       </c>
       <c r="E34" s="10"/>
       <c r="F34" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="G34" s="2"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>55</v>
+      </c>
+      <c r="B39" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A39" t="s">
-        <v>57</v>
-      </c>
-      <c r="B39" t="s">
+      <c r="B40" t="s">
         <v>62</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="A40" t="s">
-        <v>63</v>
-      </c>
-      <c r="B40" t="s">
-        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -1366,26 +1380,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1634752a-a613-4398-a360-f487231aa692">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="8e708373-a25e-443b-a8d0-0536092949a0" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EC65E7E0E531E94994381BE3B6E42323" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d474c89c2c4b816920338ad869eff1c0">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1634752a-a613-4398-a360-f487231aa692" xmlns:ns3="8e708373-a25e-443b-a8d0-0536092949a0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7b47a17d4878393dc35b05add4a78adc" ns2:_="" ns3:_="">
     <xsd:import namespace="1634752a-a613-4398-a360-f487231aa692"/>
@@ -1592,10 +1586,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1634752a-a613-4398-a360-f487231aa692">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="8e708373-a25e-443b-a8d0-0536092949a0" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6CD0A54C-38C3-4696-9E38-3A46C4CF2727}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{32255A4C-5A50-433A-AEE8-3C770C4AB65F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="1634752a-a613-4398-a360-f487231aa692"/>
+    <ds:schemaRef ds:uri="8e708373-a25e-443b-a8d0-0536092949a0"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1612,20 +1637,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{32255A4C-5A50-433A-AEE8-3C770C4AB65F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6CD0A54C-38C3-4696-9E38-3A46C4CF2727}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="1634752a-a613-4398-a360-f487231aa692"/>
-    <ds:schemaRef ds:uri="8e708373-a25e-443b-a8d0-0536092949a0"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
pin numbering and board changes
</commit_message>
<xml_diff>
--- a/tool/ESP32_Pinout.xlsx
+++ b/tool/ESP32_Pinout.xlsx
@@ -5,17 +5,18 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Files_NK\Projects\SEED25\tool\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\myspa\Projects\SEED25\tool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E30887A0-D381-4795-A5B3-D34D74A3700B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC63E5CD-9F9C-4C04-8792-EE3BC9FD93D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="1695" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="70">
   <si>
     <t>ESP32 Devkit V1 30 pin</t>
   </si>
@@ -216,18 +217,6 @@
     <t>Left Top</t>
   </si>
   <si>
-    <t>HB 1</t>
-  </si>
-  <si>
-    <t>HB 3</t>
-  </si>
-  <si>
-    <t>HB 4</t>
-  </si>
-  <si>
-    <t>HB 2</t>
-  </si>
-  <si>
     <t>(ALT) Step Step</t>
   </si>
   <si>
@@ -241,6 +230,12 @@
   </si>
   <si>
     <t>Input Only (NO PULLUP!)</t>
+  </si>
+  <si>
+    <t>HB CW</t>
+  </si>
+  <si>
+    <t>HB CCW</t>
   </si>
 </sst>
 </file>
@@ -771,20 +766,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G40"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="4" max="4" width="29.140625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="13.85546875" customWidth="1"/>
-    <col min="6" max="6" width="5.42578125" customWidth="1"/>
-    <col min="7" max="7" width="19.5703125" customWidth="1"/>
+    <col min="4" max="4" width="29.15625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="13.83984375" customWidth="1"/>
+    <col min="6" max="6" width="5.41796875" customWidth="1"/>
+    <col min="7" max="7" width="19.578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="14.7" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="29.1" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A2" s="15" t="s">
         <v>1</v>
       </c>
@@ -807,7 +802,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="11" t="s">
         <v>5</v>
       </c>
@@ -824,7 +819,7 @@
       </c>
       <c r="G3" s="11"/>
     </row>
-    <row r="4" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
@@ -841,7 +836,7 @@
       </c>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="2" t="s">
         <v>7</v>
       </c>
@@ -858,7 +853,7 @@
       </c>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="2" t="s">
         <v>8</v>
       </c>
@@ -875,7 +870,7 @@
       </c>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="2" t="s">
         <v>9</v>
       </c>
@@ -892,7 +887,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
@@ -909,7 +904,7 @@
       </c>
       <c r="G8" s="2"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="7" t="s">
         <v>11</v>
       </c>
@@ -926,7 +921,7 @@
       </c>
       <c r="G9" s="2"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="7" t="s">
         <v>12</v>
       </c>
@@ -943,7 +938,7 @@
       </c>
       <c r="G10" s="2"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="7" t="s">
         <v>13</v>
       </c>
@@ -960,7 +955,7 @@
       </c>
       <c r="G11" s="2"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="7" t="s">
         <v>14</v>
       </c>
@@ -977,7 +972,7 @@
       </c>
       <c r="G12" s="2"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="7" t="s">
         <v>15</v>
       </c>
@@ -994,7 +989,7 @@
       </c>
       <c r="G13" s="2"/>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="7" t="s">
         <v>16</v>
       </c>
@@ -1011,7 +1006,7 @@
       </c>
       <c r="G14" s="2"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="2" t="s">
         <v>17</v>
       </c>
@@ -1028,7 +1023,7 @@
       </c>
       <c r="G15" s="2"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="2" t="s">
         <v>18</v>
       </c>
@@ -1043,7 +1038,7 @@
       </c>
       <c r="G16" s="2"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="2" t="s">
         <v>19</v>
       </c>
@@ -1058,7 +1053,7 @@
       </c>
       <c r="G17" s="2"/>
     </row>
-    <row r="18" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="2" t="s">
         <v>20</v>
       </c>
@@ -1075,7 +1070,7 @@
       </c>
       <c r="G18" s="2"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="2" t="s">
         <v>22</v>
       </c>
@@ -1089,10 +1084,10 @@
         <v>55</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="2" t="s">
         <v>23</v>
       </c>
@@ -1106,10 +1101,10 @@
         <v>55</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="2" t="s">
         <v>21</v>
       </c>
@@ -1126,7 +1121,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="2" t="s">
         <v>36</v>
       </c>
@@ -1143,7 +1138,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="2" t="s">
         <v>24</v>
       </c>
@@ -1162,7 +1157,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="2" t="s">
         <v>25</v>
       </c>
@@ -1181,7 +1176,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="2" t="s">
         <v>26</v>
       </c>
@@ -1195,10 +1190,10 @@
         <v>56</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="2" t="s">
         <v>27</v>
       </c>
@@ -1212,10 +1207,10 @@
         <v>61</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="2" t="s">
         <v>28</v>
       </c>
@@ -1229,10 +1224,10 @@
         <v>58</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="2" t="s">
         <v>29</v>
       </c>
@@ -1246,10 +1241,10 @@
         <v>58</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" s="2" t="s">
         <v>30</v>
       </c>
@@ -1262,11 +1257,9 @@
       <c r="F29" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="G29" s="2" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G29" s="2"/>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="2" t="s">
         <v>31</v>
       </c>
@@ -1279,11 +1272,9 @@
       <c r="F30" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="G30" s="2" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G30" s="2"/>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="2" t="s">
         <v>32</v>
       </c>
@@ -1292,7 +1283,7 @@
       </c>
       <c r="C31" s="4"/>
       <c r="D31" s="3" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="E31" s="10"/>
       <c r="F31" s="2" t="s">
@@ -1300,7 +1291,7 @@
       </c>
       <c r="G31" s="2"/>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="2" t="s">
         <v>33</v>
       </c>
@@ -1309,7 +1300,7 @@
       </c>
       <c r="C32" s="4"/>
       <c r="D32" s="3" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="E32" s="10"/>
       <c r="F32" s="2" t="s">
@@ -1317,7 +1308,7 @@
       </c>
       <c r="G32" s="2"/>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="2" t="s">
         <v>34</v>
       </c>
@@ -1326,7 +1317,7 @@
       </c>
       <c r="C33" s="4"/>
       <c r="D33" s="3" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="E33" s="10"/>
       <c r="F33" s="2" t="s">
@@ -1334,7 +1325,7 @@
       </c>
       <c r="G33" s="2"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="2" t="s">
         <v>35</v>
       </c>
@@ -1343,7 +1334,7 @@
       </c>
       <c r="C34" s="4"/>
       <c r="D34" s="3" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="E34" s="10"/>
       <c r="F34" s="2" t="s">
@@ -1351,12 +1342,12 @@
       </c>
       <c r="G34" s="2"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" t="s">
         <v>55</v>
       </c>
@@ -1364,7 +1355,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A40" t="s">
         <v>61</v>
       </c>
@@ -1380,6 +1371,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1634752a-a613-4398-a360-f487231aa692">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="8e708373-a25e-443b-a8d0-0536092949a0" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EC65E7E0E531E94994381BE3B6E42323" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d474c89c2c4b816920338ad869eff1c0">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1634752a-a613-4398-a360-f487231aa692" xmlns:ns3="8e708373-a25e-443b-a8d0-0536092949a0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7b47a17d4878393dc35b05add4a78adc" ns2:_="" ns3:_="">
     <xsd:import namespace="1634752a-a613-4398-a360-f487231aa692"/>
@@ -1586,17 +1588,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1634752a-a613-4398-a360-f487231aa692">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="8e708373-a25e-443b-a8d0-0536092949a0" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -1607,6 +1598,17 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C2E744C2-85AC-4198-B998-4253342E25BB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="1634752a-a613-4398-a360-f487231aa692"/>
+    <ds:schemaRef ds:uri="8e708373-a25e-443b-a8d0-0536092949a0"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{32255A4C-5A50-433A-AEE8-3C770C4AB65F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1625,17 +1627,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C2E744C2-85AC-4198-B998-4253342E25BB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="1634752a-a613-4398-a360-f487231aa692"/>
-    <ds:schemaRef ds:uri="8e708373-a25e-443b-a8d0-0536092949a0"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6CD0A54C-38C3-4696-9E38-3A46C4CF2727}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Finished schematic capture and started board layout
</commit_message>
<xml_diff>
--- a/tool/ESP32_Pinout.xlsx
+++ b/tool/ESP32_Pinout.xlsx
@@ -5,18 +5,17 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\myspa\Projects\SEED25\tool\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Files_NK\Projects\SEED25\tool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC63E5CD-9F9C-4C04-8792-EE3BC9FD93D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90FB4622-50F7-474D-AB2F-4A029B0755A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38295" yWindow="1815" windowWidth="14610" windowHeight="17385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -26,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="73">
   <si>
     <t>ESP32 Devkit V1 30 pin</t>
   </si>
@@ -236,6 +235,15 @@
   </si>
   <si>
     <t>HB CCW</t>
+  </si>
+  <si>
+    <t>TOF optional Interupt</t>
+  </si>
+  <si>
+    <t>Current Sense</t>
+  </si>
+  <si>
+    <t>HB en</t>
   </si>
 </sst>
 </file>
@@ -458,15 +466,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>104114</xdr:colOff>
+      <xdr:colOff>227939</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>12840</xdr:rowOff>
+      <xdr:rowOff>3315</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>553922</xdr:colOff>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>68147</xdr:colOff>
       <xdr:row>9</xdr:row>
-      <xdr:rowOff>100440</xdr:rowOff>
+      <xdr:rowOff>90915</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -489,8 +497,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7263601" y="198370"/>
-          <a:ext cx="4286312" cy="2648200"/>
+          <a:off x="6743039" y="203340"/>
+          <a:ext cx="4107408" cy="3145125"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -766,20 +774,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G40"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="29.15625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="13.83984375" customWidth="1"/>
-    <col min="6" max="6" width="5.41796875" customWidth="1"/>
-    <col min="7" max="7" width="19.578125" customWidth="1"/>
+    <col min="4" max="4" width="29.140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="13.85546875" customWidth="1"/>
+    <col min="6" max="6" width="5.42578125" customWidth="1"/>
+    <col min="7" max="7" width="21.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="14.7" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="1" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="29.1" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="2" spans="1:7" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="15" t="s">
         <v>1</v>
       </c>
@@ -802,7 +810,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
         <v>5</v>
       </c>
@@ -819,7 +827,7 @@
       </c>
       <c r="G3" s="11"/>
     </row>
-    <row r="4" spans="1:7" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
@@ -836,7 +844,7 @@
       </c>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>7</v>
       </c>
@@ -853,7 +861,7 @@
       </c>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>8</v>
       </c>
@@ -870,7 +878,7 @@
       </c>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>9</v>
       </c>
@@ -887,7 +895,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
@@ -904,7 +912,7 @@
       </c>
       <c r="G8" s="2"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
         <v>11</v>
       </c>
@@ -921,7 +929,7 @@
       </c>
       <c r="G9" s="2"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
         <v>12</v>
       </c>
@@ -938,7 +946,7 @@
       </c>
       <c r="G10" s="2"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
         <v>13</v>
       </c>
@@ -955,7 +963,7 @@
       </c>
       <c r="G11" s="2"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
         <v>14</v>
       </c>
@@ -972,7 +980,7 @@
       </c>
       <c r="G12" s="2"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
         <v>15</v>
       </c>
@@ -989,7 +997,7 @@
       </c>
       <c r="G13" s="2"/>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
         <v>16</v>
       </c>
@@ -1006,7 +1014,7 @@
       </c>
       <c r="G14" s="2"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>17</v>
       </c>
@@ -1023,7 +1031,7 @@
       </c>
       <c r="G15" s="2"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>18</v>
       </c>
@@ -1036,9 +1044,11 @@
       <c r="F16" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="G16" s="2"/>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="G16" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>19</v>
       </c>
@@ -1053,7 +1063,7 @@
       </c>
       <c r="G17" s="2"/>
     </row>
-    <row r="18" spans="1:7" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>20</v>
       </c>
@@ -1070,7 +1080,7 @@
       </c>
       <c r="G18" s="2"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>22</v>
       </c>
@@ -1087,7 +1097,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>23</v>
       </c>
@@ -1104,7 +1114,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>21</v>
       </c>
@@ -1121,7 +1131,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>36</v>
       </c>
@@ -1138,7 +1148,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>24</v>
       </c>
@@ -1157,7 +1167,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>25</v>
       </c>
@@ -1176,7 +1186,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>26</v>
       </c>
@@ -1193,7 +1203,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>27</v>
       </c>
@@ -1210,7 +1220,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>28</v>
       </c>
@@ -1227,7 +1237,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>29</v>
       </c>
@@ -1244,7 +1254,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>30</v>
       </c>
@@ -1257,9 +1267,11 @@
       <c r="F29" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="G29" s="2"/>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="G29" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>31</v>
       </c>
@@ -1274,7 +1286,7 @@
       </c>
       <c r="G30" s="2"/>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>32</v>
       </c>
@@ -1289,9 +1301,11 @@
       <c r="F31" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="G31" s="2"/>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="G31" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>33</v>
       </c>
@@ -1308,7 +1322,7 @@
       </c>
       <c r="G32" s="2"/>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>34</v>
       </c>
@@ -1325,7 +1339,7 @@
       </c>
       <c r="G33" s="2"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>35</v>
       </c>
@@ -1342,12 +1356,12 @@
       </c>
       <c r="G34" s="2"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>55</v>
       </c>
@@ -1355,7 +1369,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>61</v>
       </c>
@@ -1371,14 +1385,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1634752a-a613-4398-a360-f487231aa692">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="8e708373-a25e-443b-a8d0-0536092949a0" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1589,21 +1601,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1634752a-a613-4398-a360-f487231aa692">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="8e708373-a25e-443b-a8d0-0536092949a0" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C2E744C2-85AC-4198-B998-4253342E25BB}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6CD0A54C-38C3-4696-9E38-3A46C4CF2727}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="1634752a-a613-4398-a360-f487231aa692"/>
-    <ds:schemaRef ds:uri="8e708373-a25e-443b-a8d0-0536092949a0"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1628,9 +1639,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6CD0A54C-38C3-4696-9E38-3A46C4CF2727}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C2E744C2-85AC-4198-B998-4253342E25BB}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="1634752a-a613-4398-a360-f487231aa692"/>
+    <ds:schemaRef ds:uri="8e708373-a25e-443b-a8d0-0536092949a0"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>